<commit_message>
feat: implement relational multi-sheet test data mapping
</commit_message>
<xml_diff>
--- a/TestData/Master_TestData.xlsx
+++ b/TestData/Master_TestData.xlsx
@@ -8,20 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saisr\Downloads\Flight_Legacy_Framework\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0C0DB4D-4B13-4564-8B91-76D5B3BF727E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1BB69BF-9154-4216-B57B-AEC4278DC5C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MasterControl" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
+    <sheet name="SearchData" sheetId="3" r:id="rId2"/>
+    <sheet name="LoginData" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="26">
   <si>
     <t>TestID</t>
   </si>
@@ -29,9 +30,6 @@
     <t>ExecutionFlowTemplate</t>
   </si>
   <si>
-    <t>Execution</t>
-  </si>
-  <si>
     <t>Username</t>
   </si>
   <si>
@@ -99,6 +97,9 @@
   </si>
   <si>
     <t>No</t>
+  </si>
+  <si>
+    <t>ExecutionFlag</t>
   </si>
 </sst>
 </file>
@@ -364,10 +365,13 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="19.90625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -375,133 +379,73 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="B2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E2" s="1" t="s">
+    </row>
+    <row r="3" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="B3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>13</v>
-      </c>
       <c r="C3" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E3" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>15</v>
-      </c>
       <c r="B4" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+      <c r="B5" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>18</v>
-      </c>
       <c r="C5" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="G5" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>21</v>
-      </c>
       <c r="B6" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="G6" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+      <c r="B7" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>24</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -510,10 +454,154 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3143AA7-45FF-46F8-8CA1-870EA82F4BF0}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="10.6328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>23</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8474CC1-798E-4C1E-B552-CA42EE506368}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>